<commit_message>
feat(buoi-03): dựng nội dung Buổi 3 vào workbook, rút gọn prompt Demo 1/2 và cập nhật file demo
- workbook: thêm đầy đủ nội dung Buổi 3 (MCP, Google Apps Script Web App, Demo 1 Dashboard, Demo 2 quản lý đơn hàng B2B); sidebar bổ sung mục lục con và đổi nhãn thành "Kết nối MCP & Google Sheets/Drive"
- rút gọn prompt Demo 1 và 3 prompt Demo 2 sang bản đơn giản, đọc dữ liệu trực tiếp qua link Google Sheets
- cập nhật 2 file Excel demo buổi 3 (Demo 1 dashboard 1 sheet, Demo 2 database 4 sheet)
- gỡ dòng .gitignore trỏ tới file Excel cũ đã tách
</commit_message>
<xml_diff>
--- a/demo-files/buoi-03/Demo 1 - Du lieu Dashboard Doanh so NovaTech.xlsx
+++ b/demo-files/buoi-03/Demo 1 - Du lieu Dashboard Doanh so NovaTech.xlsx
@@ -455,12 +455,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -518,7 +518,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1033,12 +1033,12 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>DH-2026-014</t>
+          <t>DH-2026-02-03</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Chờ thanh toán</t>
+          <t>Đã thanh toán</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Chờ thanh toán</t>
+          <t>Đã thanh toán</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1301,12 +1301,1212 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Lê Hoàng Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Chuỗi Bán lẻ Con Cưng Hà Nội</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Vũ Mai Linh</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Công ty Cổ phần Gỗ An Cường</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Trần Thị Mai</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Giao Hàng Tiết Kiệm Chi nhánh</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Custom Cloud</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>220000000</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Hoàng Minh Đức</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Viện Nghiên cứu Đào tạo Doanh nhân PTI</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Phạm Thu Thảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Tập đoàn Hóa chất Đức Giang</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Lê Hoàng Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Bóng đèn Phích nước Rạng Đông</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Vũ Mai Linh</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Chuỗi Nhà thuốc Pharmacity Miền Bắc</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Lê Hoàng Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Công ty TNHH Cơ khí Hồng Hà</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Phạm Thu Thảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Hệ thống Trường Marie Curie Hà Nội</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Trần Thị Mai</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Tập đoàn Vàng bạc Đá quý DOJI</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Custom Cloud</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>260000000</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Hùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Dược liệu Hậu Giang Chi nhánh</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Vũ Mai Linh</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Vận tải Xăng dầu VIPCO</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>130000000</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Đang xử lý</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Hoàng Minh Đức</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Tập đoàn Sơn Hải Phòng</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Phạm Thu Thảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Nhựa Tiền Phong Chi nhánh</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Lê Hoàng Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Tập đoàn Bất động sản An Phú</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>135000000</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
           <t>Chờ thanh toán</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Trần Thị Mai</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Bia Sài Gòn Miền Bắc</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Hùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Công ty Cổ phần Dệt may Nam Định</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Hùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Công ty Vận tải &amp; Kho vận Transimex</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Hoàng Minh Đức</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Khách sạn Meliá Hà Nội</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Vũ Mai Linh</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Sữa Quốc tế IDP</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Hùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Dược phẩm Pharbaco</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Phạm Thu Thảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Tổng Công ty Viglacera - CTCP</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>165000000</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>Lê Hoàng Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Công ty TNHH MTV Phân đạm Hà Bắc</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Đang xử lý</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Hoàng Minh Đức</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Chuỗi Siêu thị WinCommerce</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Custom Cloud</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>280000000</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Trần Thị Mai</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Logistics Vinalink</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Vũ Mai Linh</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP May Xuất khẩu Việt Hưng</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Đã thanh toán</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Phạm Thu Thảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Thép Pomina Hà Nội</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>120000000</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Đang xử lý</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Lê Hoàng Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Hệ thống Thẩm mỹ Thu Cúc Clinics</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Trần Thị Mai</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP Cáp điện Cadisun</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>135000000</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Chia 3 đợt</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Hùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>DH-2026-050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Công ty CP FPT Software Tuyển dụng</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khoản 100%</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Vũ Mai Linh</t>
         </is>
       </c>
     </row>

</xml_diff>